<commit_message>
Update Taj price history
</commit_message>
<xml_diff>
--- a/Taj_Price_History.xlsx
+++ b/Taj_Price_History.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -509,6 +509,38 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-07 04:42:45</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>13005</v>
+      </c>
+      <c r="C3" t="n">
+        <v>14450</v>
+      </c>
+      <c r="D3" t="n">
+        <v>13905</v>
+      </c>
+      <c r="E3" t="n">
+        <v>15450</v>
+      </c>
+      <c r="F3" t="n">
+        <v>13005</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SUPERIOR ROOM TWIN BED</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>MEMBER</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Use India time for Taj history
</commit_message>
<xml_diff>
--- a/Taj_Price_History.xlsx
+++ b/Taj_Price_History.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -480,7 +480,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-07 04:09:19</t>
+          <t>2026-09-07 09:39:19</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-09-07 04:42:45</t>
+          <t>2026-09-07 10:12:45</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -544,7 +544,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-09-07 05:11:52</t>
+          <t>2026-09-07 10:41:52</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -576,7 +576,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-09-07 05:41:55</t>
+          <t>2026-09-07 11:11:55</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -608,7 +608,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-09-07 06:17:21</t>
+          <t>2026-09-07 11:47:21</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -640,7 +640,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-09-07 06:47:07</t>
+          <t>2026-09-07 12:17:07</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -672,7 +672,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-09-07 07:14:15</t>
+          <t>2026-09-07 12:44:15</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -704,7 +704,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-09-07 07:43:13</t>
+          <t>2026-09-07 13:13:13</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -736,7 +736,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-09-07 08:13:48</t>
+          <t>2026-09-07 13:43:48</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -768,7 +768,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-09-07 08:43:13</t>
+          <t>2026-09-07 14:13:13</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -800,7 +800,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-09-07 09:13:37</t>
+          <t>2026-09-07 14:43:37</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -832,7 +832,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-09-07 09:43:20</t>
+          <t>2026-09-07 15:13:20</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -864,7 +864,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-09-07 10:12:28</t>
+          <t>2026-09-07 15:42:28</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -896,7 +896,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-09-07 10:41:33</t>
+          <t>2026-09-07 16:11:33</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -928,7 +928,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-09-07 11:12:34</t>
+          <t>2026-09-07 16:42:34</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -960,7 +960,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-09-07 11:42:13</t>
+          <t>2026-09-07 17:12:13</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -992,7 +992,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09-07 12:16:20</t>
+          <t>2026-09-07 17:46:20</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -1024,7 +1024,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09-07 12:45:59</t>
+          <t>2026-09-07 18:15:59</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1056,7 +1056,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09-07 13:13:45</t>
+          <t>2026-09-07 18:43:45</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -1088,7 +1088,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09-07 13:42:55</t>
+          <t>2026-09-07 19:12:55</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -1120,7 +1120,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09-07 14:12:59</t>
+          <t>2026-09-07 19:42:59</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -1152,7 +1152,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-09-07 14:42:19</t>
+          <t>2026-09-07 20:12:19</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -1184,7 +1184,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-09-07 15:12:02</t>
+          <t>2026-09-07 20:42:02</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -1216,7 +1216,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-09-07 15:39:51</t>
+          <t>2026-09-07 21:09:51</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -1248,7 +1248,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-09-07 15:41:55</t>
+          <t>2026-09-07 21:11:55</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1280,7 +1280,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-09-07 15:47:13</t>
+          <t>2026-09-07 21:17:13</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -1312,7 +1312,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-09-07 15:51:03</t>
+          <t>2026-09-07 21:21:03</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -1344,7 +1344,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-09-07 16:06:47</t>
+          <t>2026-09-07 21:36:47</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -1376,7 +1376,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-09-07 16:39:09</t>
+          <t>2026-09-07 22:09:09</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1408,7 +1408,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-09-07 16:50:56</t>
+          <t>2026-09-07 22:20:56</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1440,7 +1440,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-09-07 17:05:51</t>
+          <t>2026-09-07 22:35:51</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1472,7 +1472,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-09-07 17:23:29</t>
+          <t>2026-09-07 22:53:29</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1496,6 +1496,38 @@
         </is>
       </c>
       <c r="H33" t="inlineStr">
+        <is>
+          <t>MEMBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-07 23:04:12</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>12951</v>
+      </c>
+      <c r="C34" t="n">
+        <v>14390</v>
+      </c>
+      <c r="D34" t="n">
+        <v>13851</v>
+      </c>
+      <c r="E34" t="n">
+        <v>15390</v>
+      </c>
+      <c r="F34" t="n">
+        <v>12951</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>SUPERIOR ROOM TWIN BED</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>MEMBER</t>
         </is>

</xml_diff>

<commit_message>
Add Taj special price alert
</commit_message>
<xml_diff>
--- a/Taj_Price_History.xlsx
+++ b/Taj_Price_History.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1565,6 +1565,38 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-07 23:27:17</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>12951</v>
+      </c>
+      <c r="C36" t="n">
+        <v>14390</v>
+      </c>
+      <c r="D36" t="n">
+        <v>13851</v>
+      </c>
+      <c r="E36" t="n">
+        <v>15390</v>
+      </c>
+      <c r="F36" t="n">
+        <v>12951</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>SUPERIOR ROOM TWIN BED</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>MEMBER</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>